<commit_message>
se modifica para que rae y rac trabajen con coclo escolar activo, se agrega fecha de nacimiento al modelo alumno y el calculo automatico de edad con base en eso.
</commit_message>
<xml_diff>
--- a/usaer_system/rae/static/excel_templates/rae_template.xlsx
+++ b/usaer_system/rae/static/excel_templates/rae_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10824"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yoshiryquinonez/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{533AB768-6E44-7A4E-A92A-75369AD86D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724E3C94-CA74-4349-9737-7AEFB401D21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="8660" windowWidth="28800" windowHeight="15780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="26" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="74">
   <si>
     <t xml:space="preserve">ESCUELA: </t>
   </si>
@@ -252,15 +252,6 @@
   </si>
   <si>
     <t xml:space="preserve"> MÚLTIPLE (DM)</t>
-  </si>
-  <si>
-    <t>PAPELERIA FIN DE CICLO 2024/2025</t>
-  </si>
-  <si>
-    <t>EDUCACIÓN ESPECIAL</t>
-  </si>
-  <si>
-    <t>RELACIÓN DE ESCUELA POR ALUMNO</t>
   </si>
   <si>
     <t xml:space="preserve">LUGAR:   </t>
@@ -969,7 +960,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="6" applyFont="1"/>
@@ -1201,10 +1192,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1227,66 +1214,35 @@
     <xf numFmtId="49" fontId="5" fillId="4" borderId="22" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="9" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="9" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="45" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="4" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="44" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="19" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="10" fillId="3" borderId="19" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="4" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="19" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="8" fillId="3" borderId="43" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="8" fillId="3" borderId="41" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1298,32 +1254,63 @@
     <xf numFmtId="49" fontId="10" fillId="3" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="10" fillId="3" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="21" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="1" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="45" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="19" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="4" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="44" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="19" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="19" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="6" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="9" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="9" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="2" borderId="4" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2698,35 +2685,33 @@
       <c r="AR1" s="39"/>
     </row>
     <row r="2" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="145" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" s="146"/>
-      <c r="C2" s="146"/>
-      <c r="D2" s="146"/>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="146"/>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
-      <c r="K2" s="146"/>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
-      <c r="O2" s="146"/>
-      <c r="P2" s="146"/>
-      <c r="Q2" s="146"/>
-      <c r="R2" s="146"/>
-      <c r="S2" s="146"/>
-      <c r="T2" s="146"/>
-      <c r="U2" s="146"/>
-      <c r="V2" s="146"/>
-      <c r="W2" s="146"/>
-      <c r="X2" s="146"/>
-      <c r="Y2" s="146"/>
-      <c r="Z2" s="146"/>
-      <c r="AA2" s="146"/>
+      <c r="A2" s="101"/>
+      <c r="B2" s="102"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="102"/>
+      <c r="K2" s="102"/>
+      <c r="L2" s="102"/>
+      <c r="M2" s="102"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="102"/>
+      <c r="P2" s="102"/>
+      <c r="Q2" s="102"/>
+      <c r="R2" s="102"/>
+      <c r="S2" s="102"/>
+      <c r="T2" s="102"/>
+      <c r="U2" s="102"/>
+      <c r="V2" s="102"/>
+      <c r="W2" s="102"/>
+      <c r="X2" s="102"/>
+      <c r="Y2" s="102"/>
+      <c r="Z2" s="102"/>
+      <c r="AA2" s="102"/>
       <c r="AB2" s="39"/>
       <c r="AC2" s="39"/>
       <c r="AD2" s="39"/>
@@ -2746,35 +2731,33 @@
       <c r="AR2" s="39"/>
     </row>
     <row r="3" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="145" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="146"/>
-      <c r="C3" s="146"/>
-      <c r="D3" s="146"/>
-      <c r="E3" s="146"/>
-      <c r="F3" s="146"/>
-      <c r="G3" s="146"/>
-      <c r="H3" s="146"/>
-      <c r="I3" s="146"/>
-      <c r="J3" s="146"/>
-      <c r="K3" s="146"/>
-      <c r="L3" s="146"/>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="146"/>
-      <c r="P3" s="146"/>
-      <c r="Q3" s="146"/>
-      <c r="R3" s="146"/>
-      <c r="S3" s="146"/>
-      <c r="T3" s="146"/>
-      <c r="U3" s="146"/>
-      <c r="V3" s="146"/>
-      <c r="W3" s="146"/>
-      <c r="X3" s="146"/>
-      <c r="Y3" s="146"/>
-      <c r="Z3" s="146"/>
-      <c r="AA3" s="146"/>
+      <c r="A3" s="101"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102"/>
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="102"/>
+      <c r="R3" s="102"/>
+      <c r="S3" s="102"/>
+      <c r="T3" s="102"/>
+      <c r="U3" s="102"/>
+      <c r="V3" s="102"/>
+      <c r="W3" s="102"/>
+      <c r="X3" s="102"/>
+      <c r="Y3" s="102"/>
+      <c r="Z3" s="102"/>
+      <c r="AA3" s="102"/>
       <c r="AB3" s="39"/>
       <c r="AC3" s="39"/>
       <c r="AD3" s="39"/>
@@ -2794,35 +2777,33 @@
       <c r="AR3" s="39"/>
     </row>
     <row r="4" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="145" t="s">
-        <v>75</v>
-      </c>
-      <c r="B4" s="146"/>
-      <c r="C4" s="146"/>
-      <c r="D4" s="146"/>
-      <c r="E4" s="146"/>
-      <c r="F4" s="146"/>
-      <c r="G4" s="146"/>
-      <c r="H4" s="146"/>
-      <c r="I4" s="146"/>
-      <c r="J4" s="146"/>
-      <c r="K4" s="146"/>
-      <c r="L4" s="146"/>
-      <c r="M4" s="146"/>
-      <c r="N4" s="146"/>
-      <c r="O4" s="146"/>
-      <c r="P4" s="146"/>
-      <c r="Q4" s="146"/>
-      <c r="R4" s="146"/>
-      <c r="S4" s="146"/>
-      <c r="T4" s="146"/>
-      <c r="U4" s="146"/>
-      <c r="V4" s="146"/>
-      <c r="W4" s="146"/>
-      <c r="X4" s="146"/>
-      <c r="Y4" s="146"/>
-      <c r="Z4" s="146"/>
-      <c r="AA4" s="146"/>
+      <c r="A4" s="101"/>
+      <c r="B4" s="102"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="102"/>
+      <c r="E4" s="102"/>
+      <c r="F4" s="102"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="102"/>
+      <c r="I4" s="102"/>
+      <c r="J4" s="102"/>
+      <c r="K4" s="102"/>
+      <c r="L4" s="102"/>
+      <c r="M4" s="102"/>
+      <c r="N4" s="102"/>
+      <c r="O4" s="102"/>
+      <c r="P4" s="102"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="102"/>
+      <c r="S4" s="102"/>
+      <c r="T4" s="102"/>
+      <c r="U4" s="102"/>
+      <c r="V4" s="102"/>
+      <c r="W4" s="102"/>
+      <c r="X4" s="102"/>
+      <c r="Y4" s="102"/>
+      <c r="Z4" s="102"/>
+      <c r="AA4" s="102"/>
       <c r="AB4" s="39"/>
       <c r="AC4" s="39"/>
       <c r="AD4" s="39"/>
@@ -2893,49 +2874,49 @@
       <c r="C6" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="124"/>
-      <c r="E6" s="147"/>
-      <c r="F6" s="147"/>
-      <c r="G6" s="147"/>
-      <c r="H6" s="147"/>
-      <c r="I6" s="147"/>
-      <c r="J6" s="147"/>
-      <c r="K6" s="147"/>
-      <c r="L6" s="147"/>
-      <c r="M6" s="147"/>
-      <c r="N6" s="147"/>
-      <c r="O6" s="147"/>
-      <c r="P6" s="147"/>
-      <c r="Q6" s="147"/>
-      <c r="R6" s="147"/>
-      <c r="S6" s="147"/>
-      <c r="T6" s="147"/>
-      <c r="U6" s="147"/>
-      <c r="V6" s="147"/>
-      <c r="W6" s="147"/>
-      <c r="X6" s="147"/>
-      <c r="Y6" s="147"/>
-      <c r="Z6" s="147"/>
-      <c r="AA6" s="148"/>
+      <c r="D6" s="103"/>
+      <c r="E6" s="104"/>
+      <c r="F6" s="104"/>
+      <c r="G6" s="104"/>
+      <c r="H6" s="104"/>
+      <c r="I6" s="104"/>
+      <c r="J6" s="104"/>
+      <c r="K6" s="104"/>
+      <c r="L6" s="104"/>
+      <c r="M6" s="104"/>
+      <c r="N6" s="104"/>
+      <c r="O6" s="104"/>
+      <c r="P6" s="104"/>
+      <c r="Q6" s="104"/>
+      <c r="R6" s="104"/>
+      <c r="S6" s="104"/>
+      <c r="T6" s="104"/>
+      <c r="U6" s="104"/>
+      <c r="V6" s="104"/>
+      <c r="W6" s="104"/>
+      <c r="X6" s="104"/>
+      <c r="Y6" s="104"/>
+      <c r="Z6" s="104"/>
+      <c r="AA6" s="105"/>
       <c r="AB6" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="AC6" s="124"/>
-      <c r="AD6" s="104"/>
-      <c r="AE6" s="104"/>
-      <c r="AF6" s="104"/>
-      <c r="AG6" s="104"/>
-      <c r="AH6" s="104"/>
-      <c r="AI6" s="104"/>
-      <c r="AJ6" s="104"/>
-      <c r="AK6" s="104"/>
-      <c r="AL6" s="104"/>
-      <c r="AM6" s="104"/>
-      <c r="AN6" s="104"/>
-      <c r="AO6" s="104"/>
-      <c r="AP6" s="104"/>
-      <c r="AQ6" s="104"/>
-      <c r="AR6" s="105"/>
+      <c r="AC6" s="103"/>
+      <c r="AD6" s="106"/>
+      <c r="AE6" s="106"/>
+      <c r="AF6" s="106"/>
+      <c r="AG6" s="106"/>
+      <c r="AH6" s="106"/>
+      <c r="AI6" s="106"/>
+      <c r="AJ6" s="106"/>
+      <c r="AK6" s="106"/>
+      <c r="AL6" s="106"/>
+      <c r="AM6" s="106"/>
+      <c r="AN6" s="106"/>
+      <c r="AO6" s="106"/>
+      <c r="AP6" s="106"/>
+      <c r="AQ6" s="106"/>
+      <c r="AR6" s="107"/>
     </row>
     <row r="7" spans="1:44" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
@@ -2989,16 +2970,16 @@
       <c r="C8" s="61" t="s">
         <v>61</v>
       </c>
-      <c r="D8" s="124"/>
-      <c r="E8" s="104"/>
-      <c r="F8" s="105"/>
+      <c r="D8" s="103"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="107"/>
       <c r="G8" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="H8" s="124"/>
-      <c r="I8" s="104"/>
-      <c r="J8" s="104"/>
-      <c r="K8" s="105"/>
+      <c r="H8" s="103"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="106"/>
+      <c r="K8" s="107"/>
       <c r="L8" s="60"/>
       <c r="M8" s="82"/>
       <c r="N8" s="12" t="s">
@@ -3007,35 +2988,35 @@
       <c r="O8" s="82"/>
       <c r="P8" s="81"/>
       <c r="Q8" s="80"/>
-      <c r="R8" s="124"/>
-      <c r="S8" s="104"/>
-      <c r="T8" s="104"/>
-      <c r="U8" s="104"/>
-      <c r="V8" s="104"/>
-      <c r="W8" s="104"/>
-      <c r="X8" s="104"/>
-      <c r="Y8" s="104"/>
-      <c r="Z8" s="104"/>
-      <c r="AA8" s="105"/>
+      <c r="R8" s="103"/>
+      <c r="S8" s="106"/>
+      <c r="T8" s="106"/>
+      <c r="U8" s="106"/>
+      <c r="V8" s="106"/>
+      <c r="W8" s="106"/>
+      <c r="X8" s="106"/>
+      <c r="Y8" s="106"/>
+      <c r="Z8" s="106"/>
+      <c r="AA8" s="107"/>
       <c r="AB8" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="AC8" s="124"/>
-      <c r="AD8" s="104"/>
-      <c r="AE8" s="104"/>
-      <c r="AF8" s="104"/>
-      <c r="AG8" s="104"/>
-      <c r="AH8" s="104"/>
-      <c r="AI8" s="104"/>
-      <c r="AJ8" s="104"/>
-      <c r="AK8" s="104"/>
-      <c r="AL8" s="104"/>
-      <c r="AM8" s="104"/>
-      <c r="AN8" s="104"/>
-      <c r="AO8" s="104"/>
-      <c r="AP8" s="104"/>
-      <c r="AQ8" s="104"/>
-      <c r="AR8" s="105"/>
+      <c r="AC8" s="103"/>
+      <c r="AD8" s="106"/>
+      <c r="AE8" s="106"/>
+      <c r="AF8" s="106"/>
+      <c r="AG8" s="106"/>
+      <c r="AH8" s="106"/>
+      <c r="AI8" s="106"/>
+      <c r="AJ8" s="106"/>
+      <c r="AK8" s="106"/>
+      <c r="AL8" s="106"/>
+      <c r="AM8" s="106"/>
+      <c r="AN8" s="106"/>
+      <c r="AO8" s="106"/>
+      <c r="AP8" s="106"/>
+      <c r="AQ8" s="106"/>
+      <c r="AR8" s="107"/>
     </row>
     <row r="9" spans="1:44" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9"/>
@@ -3089,37 +3070,37 @@
       <c r="C10" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="124"/>
-      <c r="E10" s="104"/>
-      <c r="F10" s="104"/>
-      <c r="G10" s="104"/>
-      <c r="H10" s="104"/>
-      <c r="I10" s="104"/>
-      <c r="J10" s="104"/>
-      <c r="K10" s="104"/>
-      <c r="L10" s="104"/>
-      <c r="M10" s="104"/>
-      <c r="N10" s="104"/>
-      <c r="O10" s="104"/>
-      <c r="P10" s="104"/>
-      <c r="Q10" s="104"/>
-      <c r="R10" s="104"/>
-      <c r="S10" s="104"/>
-      <c r="T10" s="104"/>
-      <c r="U10" s="104"/>
-      <c r="V10" s="104"/>
-      <c r="W10" s="104"/>
-      <c r="X10" s="104"/>
-      <c r="Y10" s="104"/>
-      <c r="Z10" s="104"/>
-      <c r="AA10" s="105"/>
-      <c r="AB10" s="141" t="s">
+      <c r="D10" s="103"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="106"/>
+      <c r="J10" s="106"/>
+      <c r="K10" s="106"/>
+      <c r="L10" s="106"/>
+      <c r="M10" s="106"/>
+      <c r="N10" s="106"/>
+      <c r="O10" s="106"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
+      <c r="R10" s="106"/>
+      <c r="S10" s="106"/>
+      <c r="T10" s="106"/>
+      <c r="U10" s="106"/>
+      <c r="V10" s="106"/>
+      <c r="W10" s="106"/>
+      <c r="X10" s="106"/>
+      <c r="Y10" s="106"/>
+      <c r="Z10" s="106"/>
+      <c r="AA10" s="107"/>
+      <c r="AB10" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="AC10" s="143" t="s">
+      <c r="AC10" s="110" t="s">
         <v>7</v>
       </c>
-      <c r="AD10" s="128"/>
+      <c r="AD10" s="111"/>
       <c r="AE10" s="75" t="s">
         <v>48</v>
       </c>
@@ -3129,10 +3110,10 @@
       <c r="AG10" s="75" t="s">
         <v>55</v>
       </c>
-      <c r="AH10" s="127" t="s">
+      <c r="AH10" s="114" t="s">
         <v>8</v>
       </c>
-      <c r="AI10" s="128"/>
+      <c r="AI10" s="111"/>
       <c r="AJ10" s="75" t="s">
         <v>48</v>
       </c>
@@ -3142,11 +3123,11 @@
       <c r="AL10" s="73" t="s">
         <v>55</v>
       </c>
-      <c r="AM10" s="131" t="s">
+      <c r="AM10" s="116" t="s">
         <v>9</v>
       </c>
-      <c r="AN10" s="132"/>
-      <c r="AO10" s="133"/>
+      <c r="AN10" s="117"/>
+      <c r="AO10" s="118"/>
       <c r="AP10" s="74" t="s">
         <v>48</v>
       </c>
@@ -3185,20 +3166,20 @@
       <c r="Y11" s="68"/>
       <c r="Z11" s="68"/>
       <c r="AA11" s="68"/>
-      <c r="AB11" s="142"/>
-      <c r="AC11" s="144"/>
-      <c r="AD11" s="130"/>
+      <c r="AB11" s="109"/>
+      <c r="AC11" s="112"/>
+      <c r="AD11" s="113"/>
       <c r="AE11" s="67"/>
       <c r="AF11" s="66"/>
       <c r="AG11" s="18"/>
-      <c r="AH11" s="129"/>
-      <c r="AI11" s="130"/>
+      <c r="AH11" s="115"/>
+      <c r="AI11" s="113"/>
       <c r="AJ11" s="67"/>
       <c r="AK11" s="66"/>
       <c r="AL11" s="65"/>
-      <c r="AM11" s="134"/>
-      <c r="AN11" s="135"/>
-      <c r="AO11" s="136"/>
+      <c r="AM11" s="119"/>
+      <c r="AN11" s="120"/>
+      <c r="AO11" s="121"/>
       <c r="AP11" s="64"/>
       <c r="AQ11" s="63"/>
       <c r="AR11" s="62"/>
@@ -3209,32 +3190,32 @@
       <c r="C12" s="61" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="120"/>
-      <c r="E12" s="104"/>
-      <c r="F12" s="104"/>
-      <c r="G12" s="105"/>
+      <c r="D12" s="132"/>
+      <c r="E12" s="106"/>
+      <c r="F12" s="106"/>
+      <c r="G12" s="107"/>
       <c r="H12" s="60"/>
-      <c r="I12" s="121" t="s">
+      <c r="I12" s="133" t="s">
         <v>3</v>
       </c>
-      <c r="J12" s="108"/>
-      <c r="K12" s="108"/>
-      <c r="L12" s="108"/>
-      <c r="M12" s="108"/>
-      <c r="N12" s="108"/>
-      <c r="O12" s="108"/>
-      <c r="P12" s="108"/>
-      <c r="Q12" s="122"/>
-      <c r="R12" s="124"/>
-      <c r="S12" s="104"/>
-      <c r="T12" s="104"/>
-      <c r="U12" s="104"/>
-      <c r="V12" s="104"/>
-      <c r="W12" s="104"/>
-      <c r="X12" s="104"/>
-      <c r="Y12" s="104"/>
-      <c r="Z12" s="104"/>
-      <c r="AA12" s="105"/>
+      <c r="J12" s="134"/>
+      <c r="K12" s="134"/>
+      <c r="L12" s="134"/>
+      <c r="M12" s="134"/>
+      <c r="N12" s="134"/>
+      <c r="O12" s="134"/>
+      <c r="P12" s="134"/>
+      <c r="Q12" s="135"/>
+      <c r="R12" s="103"/>
+      <c r="S12" s="106"/>
+      <c r="T12" s="106"/>
+      <c r="U12" s="106"/>
+      <c r="V12" s="106"/>
+      <c r="W12" s="106"/>
+      <c r="X12" s="106"/>
+      <c r="Y12" s="106"/>
+      <c r="Z12" s="106"/>
+      <c r="AA12" s="107"/>
       <c r="AB12" s="59"/>
       <c r="AC12" s="3"/>
       <c r="AD12" s="3"/>
@@ -3305,51 +3286,51 @@
       <c r="C14" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="120"/>
-      <c r="E14" s="104"/>
-      <c r="F14" s="104"/>
-      <c r="G14" s="104"/>
-      <c r="H14" s="104"/>
-      <c r="I14" s="104"/>
-      <c r="J14" s="104"/>
-      <c r="K14" s="104"/>
-      <c r="L14" s="104"/>
-      <c r="M14" s="104"/>
-      <c r="N14" s="104"/>
-      <c r="O14" s="104"/>
-      <c r="P14" s="104"/>
-      <c r="Q14" s="104"/>
-      <c r="R14" s="104"/>
-      <c r="S14" s="104"/>
-      <c r="T14" s="104"/>
-      <c r="U14" s="104"/>
-      <c r="V14" s="104"/>
-      <c r="W14" s="104"/>
-      <c r="X14" s="104"/>
-      <c r="Y14" s="104"/>
-      <c r="Z14" s="104"/>
-      <c r="AA14" s="105"/>
+      <c r="D14" s="132"/>
+      <c r="E14" s="106"/>
+      <c r="F14" s="106"/>
+      <c r="G14" s="106"/>
+      <c r="H14" s="106"/>
+      <c r="I14" s="106"/>
+      <c r="J14" s="106"/>
+      <c r="K14" s="106"/>
+      <c r="L14" s="106"/>
+      <c r="M14" s="106"/>
+      <c r="N14" s="106"/>
+      <c r="O14" s="106"/>
+      <c r="P14" s="106"/>
+      <c r="Q14" s="106"/>
+      <c r="R14" s="106"/>
+      <c r="S14" s="106"/>
+      <c r="T14" s="106"/>
+      <c r="U14" s="106"/>
+      <c r="V14" s="106"/>
+      <c r="W14" s="106"/>
+      <c r="X14" s="106"/>
+      <c r="Y14" s="106"/>
+      <c r="Z14" s="106"/>
+      <c r="AA14" s="107"/>
       <c r="AB14" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="AC14" s="119" t="s">
+      <c r="AC14" s="141" t="s">
         <v>50</v>
       </c>
-      <c r="AD14" s="112"/>
-      <c r="AE14" s="112"/>
-      <c r="AF14" s="116"/>
-      <c r="AG14" s="111"/>
-      <c r="AH14" s="112"/>
-      <c r="AI14" s="116"/>
+      <c r="AD14" s="125"/>
+      <c r="AE14" s="125"/>
+      <c r="AF14" s="127"/>
+      <c r="AG14" s="140"/>
+      <c r="AH14" s="125"/>
+      <c r="AI14" s="127"/>
       <c r="AJ14" s="49"/>
-      <c r="AK14" s="119" t="s">
+      <c r="AK14" s="141" t="s">
         <v>51</v>
       </c>
-      <c r="AL14" s="112"/>
-      <c r="AM14" s="112"/>
-      <c r="AN14" s="116"/>
-      <c r="AO14" s="111"/>
-      <c r="AP14" s="112"/>
+      <c r="AL14" s="125"/>
+      <c r="AM14" s="125"/>
+      <c r="AN14" s="127"/>
+      <c r="AO14" s="140"/>
+      <c r="AP14" s="125"/>
       <c r="AQ14" s="48"/>
       <c r="AR14" s="47"/>
     </row>
@@ -3401,241 +3382,241 @@
     </row>
     <row r="16" spans="1:44" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="21"/>
-      <c r="B16" s="113" t="s">
+      <c r="B16" s="136" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="113" t="s">
+      <c r="C16" s="136" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="123" t="s">
+      <c r="D16" s="137" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="123" t="s">
+      <c r="E16" s="137" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="123" t="s">
+      <c r="F16" s="137" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="113" t="s">
+      <c r="G16" s="136" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="126" t="s">
+      <c r="H16" s="124" t="s">
         <v>56</v>
       </c>
-      <c r="I16" s="112"/>
-      <c r="J16" s="112"/>
-      <c r="K16" s="112"/>
-      <c r="L16" s="112"/>
-      <c r="M16" s="112"/>
-      <c r="N16" s="112"/>
-      <c r="O16" s="112"/>
-      <c r="P16" s="112"/>
-      <c r="Q16" s="112"/>
-      <c r="R16" s="112"/>
-      <c r="S16" s="112"/>
-      <c r="T16" s="112"/>
-      <c r="U16" s="112"/>
-      <c r="V16" s="112"/>
-      <c r="W16" s="112"/>
-      <c r="X16" s="112"/>
-      <c r="Y16" s="112"/>
-      <c r="Z16" s="112"/>
-      <c r="AA16" s="112"/>
-      <c r="AB16" s="116"/>
-      <c r="AC16" s="126" t="s">
+      <c r="I16" s="125"/>
+      <c r="J16" s="125"/>
+      <c r="K16" s="125"/>
+      <c r="L16" s="125"/>
+      <c r="M16" s="125"/>
+      <c r="N16" s="125"/>
+      <c r="O16" s="125"/>
+      <c r="P16" s="125"/>
+      <c r="Q16" s="125"/>
+      <c r="R16" s="125"/>
+      <c r="S16" s="125"/>
+      <c r="T16" s="125"/>
+      <c r="U16" s="125"/>
+      <c r="V16" s="125"/>
+      <c r="W16" s="125"/>
+      <c r="X16" s="125"/>
+      <c r="Y16" s="125"/>
+      <c r="Z16" s="125"/>
+      <c r="AA16" s="125"/>
+      <c r="AB16" s="127"/>
+      <c r="AC16" s="124" t="s">
         <v>18</v>
       </c>
-      <c r="AD16" s="112"/>
-      <c r="AE16" s="112"/>
-      <c r="AF16" s="112"/>
-      <c r="AG16" s="112"/>
-      <c r="AH16" s="112"/>
-      <c r="AI16" s="112"/>
-      <c r="AJ16" s="112"/>
-      <c r="AK16" s="138" t="s">
+      <c r="AD16" s="125"/>
+      <c r="AE16" s="125"/>
+      <c r="AF16" s="125"/>
+      <c r="AG16" s="125"/>
+      <c r="AH16" s="125"/>
+      <c r="AI16" s="125"/>
+      <c r="AJ16" s="125"/>
+      <c r="AK16" s="126" t="s">
         <v>62</v>
       </c>
-      <c r="AL16" s="112"/>
-      <c r="AM16" s="112"/>
-      <c r="AN16" s="112"/>
-      <c r="AO16" s="112"/>
-      <c r="AP16" s="112"/>
-      <c r="AQ16" s="112"/>
-      <c r="AR16" s="116"/>
+      <c r="AL16" s="125"/>
+      <c r="AM16" s="125"/>
+      <c r="AN16" s="125"/>
+      <c r="AO16" s="125"/>
+      <c r="AP16" s="125"/>
+      <c r="AQ16" s="125"/>
+      <c r="AR16" s="127"/>
     </row>
     <row r="17" spans="1:44" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="21"/>
-      <c r="B17" s="114"/>
-      <c r="C17" s="114"/>
-      <c r="D17" s="114"/>
-      <c r="E17" s="114"/>
-      <c r="F17" s="114"/>
-      <c r="G17" s="114"/>
-      <c r="H17" s="125" t="s">
+      <c r="B17" s="129"/>
+      <c r="C17" s="129"/>
+      <c r="D17" s="129"/>
+      <c r="E17" s="129"/>
+      <c r="F17" s="129"/>
+      <c r="G17" s="129"/>
+      <c r="H17" s="138" t="s">
         <v>20</v>
       </c>
-      <c r="I17" s="112"/>
-      <c r="J17" s="112"/>
-      <c r="K17" s="112"/>
-      <c r="L17" s="112"/>
-      <c r="M17" s="112"/>
-      <c r="N17" s="112"/>
-      <c r="O17" s="112"/>
-      <c r="P17" s="112"/>
-      <c r="Q17" s="116"/>
-      <c r="R17" s="115" t="s">
+      <c r="I17" s="125"/>
+      <c r="J17" s="125"/>
+      <c r="K17" s="125"/>
+      <c r="L17" s="125"/>
+      <c r="M17" s="125"/>
+      <c r="N17" s="125"/>
+      <c r="O17" s="125"/>
+      <c r="P17" s="125"/>
+      <c r="Q17" s="127"/>
+      <c r="R17" s="139" t="s">
         <v>21</v>
       </c>
-      <c r="S17" s="112"/>
-      <c r="T17" s="116"/>
-      <c r="U17" s="115" t="s">
+      <c r="S17" s="125"/>
+      <c r="T17" s="127"/>
+      <c r="U17" s="139" t="s">
         <v>22</v>
       </c>
-      <c r="V17" s="116"/>
-      <c r="W17" s="115" t="s">
+      <c r="V17" s="127"/>
+      <c r="W17" s="139" t="s">
         <v>23</v>
       </c>
-      <c r="X17" s="112"/>
-      <c r="Y17" s="112"/>
-      <c r="Z17" s="112"/>
-      <c r="AA17" s="116"/>
-      <c r="AB17" s="99" t="s">
+      <c r="X17" s="125"/>
+      <c r="Y17" s="125"/>
+      <c r="Z17" s="125"/>
+      <c r="AA17" s="127"/>
+      <c r="AB17" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="AC17" s="117" t="s">
+      <c r="AC17" s="131" t="s">
         <v>24</v>
       </c>
-      <c r="AD17" s="117" t="s">
+      <c r="AD17" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="AE17" s="117" t="s">
+      <c r="AE17" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="AF17" s="117" t="s">
+      <c r="AF17" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="AG17" s="117" t="s">
+      <c r="AG17" s="131" t="s">
         <v>28</v>
       </c>
-      <c r="AH17" s="117"/>
-      <c r="AI17" s="117" t="s">
+      <c r="AH17" s="131"/>
+      <c r="AI17" s="131" t="s">
         <v>29</v>
       </c>
-      <c r="AJ17" s="117" t="s">
+      <c r="AJ17" s="131" t="s">
         <v>30</v>
       </c>
-      <c r="AK17" s="102"/>
-      <c r="AL17" s="140" t="s">
+      <c r="AK17" s="100"/>
+      <c r="AL17" s="130" t="s">
         <v>31</v>
       </c>
-      <c r="AM17" s="130"/>
-      <c r="AN17" s="137" t="s">
+      <c r="AM17" s="113"/>
+      <c r="AN17" s="122" t="s">
         <v>32</v>
       </c>
-      <c r="AO17" s="137" t="s">
+      <c r="AO17" s="122" t="s">
         <v>33</v>
       </c>
-      <c r="AP17" s="137" t="s">
+      <c r="AP17" s="122" t="s">
         <v>34</v>
       </c>
-      <c r="AQ17" s="137" t="s">
+      <c r="AQ17" s="122" t="s">
         <v>35</v>
       </c>
-      <c r="AR17" s="139" t="s">
+      <c r="AR17" s="128" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:44" ht="128.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="21"/>
-      <c r="B18" s="114"/>
-      <c r="C18" s="114"/>
-      <c r="D18" s="114"/>
-      <c r="E18" s="114"/>
-      <c r="F18" s="114"/>
-      <c r="G18" s="114"/>
-      <c r="H18" s="101" t="s">
+      <c r="B18" s="129"/>
+      <c r="C18" s="129"/>
+      <c r="D18" s="129"/>
+      <c r="E18" s="129"/>
+      <c r="F18" s="129"/>
+      <c r="G18" s="129"/>
+      <c r="H18" s="99" t="s">
         <v>57</v>
       </c>
-      <c r="I18" s="100" t="s">
+      <c r="I18" s="98" t="s">
         <v>58</v>
       </c>
-      <c r="J18" s="100" t="s">
+      <c r="J18" s="98" t="s">
         <v>59</v>
       </c>
-      <c r="K18" s="100" t="s">
+      <c r="K18" s="98" t="s">
         <v>60</v>
       </c>
-      <c r="L18" s="100" t="s">
+      <c r="L18" s="98" t="s">
         <v>36</v>
       </c>
-      <c r="M18" s="100" t="s">
+      <c r="M18" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="N18" s="100" t="s">
+      <c r="N18" s="98" t="s">
         <v>69</v>
       </c>
-      <c r="O18" s="100" t="s">
+      <c r="O18" s="98" t="s">
         <v>70</v>
       </c>
-      <c r="P18" s="100" t="s">
+      <c r="P18" s="98" t="s">
         <v>71</v>
       </c>
-      <c r="Q18" s="100" t="s">
+      <c r="Q18" s="98" t="s">
         <v>72</v>
       </c>
-      <c r="R18" s="100" t="s">
+      <c r="R18" s="98" t="s">
         <v>63</v>
       </c>
-      <c r="S18" s="100" t="s">
+      <c r="S18" s="98" t="s">
         <v>64</v>
       </c>
-      <c r="T18" s="100" t="s">
+      <c r="T18" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="U18" s="100" t="s">
+      <c r="U18" s="98" t="s">
         <v>66</v>
       </c>
-      <c r="V18" s="100" t="s">
+      <c r="V18" s="98" t="s">
         <v>67</v>
       </c>
-      <c r="W18" s="100" t="s">
+      <c r="W18" s="98" t="s">
         <v>37</v>
       </c>
-      <c r="X18" s="100" t="s">
+      <c r="X18" s="98" t="s">
         <v>38</v>
       </c>
-      <c r="Y18" s="100" t="s">
+      <c r="Y18" s="98" t="s">
         <v>39</v>
       </c>
-      <c r="Z18" s="100" t="s">
+      <c r="Z18" s="98" t="s">
         <v>40</v>
       </c>
-      <c r="AA18" s="100" t="s">
+      <c r="AA18" s="98" t="s">
         <v>41</v>
       </c>
-      <c r="AB18" s="99" t="s">
+      <c r="AB18" s="97" t="s">
         <v>42</v>
       </c>
-      <c r="AC18" s="118"/>
-      <c r="AD18" s="118"/>
-      <c r="AE18" s="118"/>
-      <c r="AF18" s="118"/>
-      <c r="AG18" s="118"/>
-      <c r="AH18" s="118"/>
-      <c r="AI18" s="118"/>
-      <c r="AJ18" s="114"/>
-      <c r="AK18" s="98"/>
-      <c r="AL18" s="97" t="s">
+      <c r="AC18" s="123"/>
+      <c r="AD18" s="123"/>
+      <c r="AE18" s="123"/>
+      <c r="AF18" s="123"/>
+      <c r="AG18" s="123"/>
+      <c r="AH18" s="123"/>
+      <c r="AI18" s="123"/>
+      <c r="AJ18" s="129"/>
+      <c r="AK18" s="96"/>
+      <c r="AL18" s="95" t="s">
         <v>43</v>
       </c>
-      <c r="AM18" s="97" t="s">
+      <c r="AM18" s="95" t="s">
         <v>44</v>
       </c>
-      <c r="AN18" s="114"/>
-      <c r="AO18" s="114"/>
-      <c r="AP18" s="118"/>
-      <c r="AQ18" s="118"/>
-      <c r="AR18" s="114"/>
+      <c r="AN18" s="129"/>
+      <c r="AO18" s="129"/>
+      <c r="AP18" s="123"/>
+      <c r="AQ18" s="123"/>
+      <c r="AR18" s="129"/>
     </row>
     <row r="19" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A19" s="36"/>
@@ -3693,7 +3674,7 @@
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
-      <c r="F20" s="96"/>
+      <c r="F20" s="94"/>
       <c r="G20" s="15"/>
       <c r="H20" s="17"/>
       <c r="I20" s="35"/>
@@ -3789,7 +3770,7 @@
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
-      <c r="F22" s="96"/>
+      <c r="F22" s="94"/>
       <c r="G22" s="15"/>
       <c r="H22" s="17"/>
       <c r="I22" s="35"/>
@@ -4211,7 +4192,7 @@
       <c r="AO30" s="16"/>
       <c r="AP30" s="25"/>
       <c r="AQ30" s="16"/>
-      <c r="AR30" s="95"/>
+      <c r="AR30" s="93"/>
     </row>
     <row r="31" spans="1:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="21"/>
@@ -4661,7 +4642,7 @@
       <c r="K40" s="23"/>
       <c r="L40" s="23"/>
       <c r="M40" s="23"/>
-      <c r="N40" s="94"/>
+      <c r="N40" s="23"/>
       <c r="O40" s="17"/>
       <c r="P40" s="23"/>
       <c r="Q40" s="23"/>
@@ -4709,7 +4690,7 @@
       <c r="K41" s="23"/>
       <c r="L41" s="23"/>
       <c r="M41" s="23"/>
-      <c r="N41" s="94"/>
+      <c r="N41" s="23"/>
       <c r="O41" s="17"/>
       <c r="P41" s="23"/>
       <c r="Q41" s="23"/>
@@ -4757,7 +4738,7 @@
       <c r="K42" s="17"/>
       <c r="L42" s="17"/>
       <c r="M42" s="17"/>
-      <c r="N42" s="93"/>
+      <c r="N42" s="23"/>
       <c r="O42" s="17"/>
       <c r="P42" s="17"/>
       <c r="Q42" s="17"/>
@@ -4805,7 +4786,7 @@
       <c r="K43" s="17"/>
       <c r="L43" s="17"/>
       <c r="M43" s="17"/>
-      <c r="N43" s="17"/>
+      <c r="N43" s="23"/>
       <c r="O43" s="17"/>
       <c r="P43" s="17"/>
       <c r="Q43" s="17"/>
@@ -6354,13 +6335,13 @@
     </row>
     <row r="76" spans="2:44" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B76" s="13"/>
-      <c r="C76" s="103" t="s">
-        <v>76</v>
+      <c r="C76" s="142" t="s">
+        <v>73</v>
       </c>
-      <c r="D76" s="104"/>
-      <c r="E76" s="104"/>
-      <c r="F76" s="104"/>
-      <c r="G76" s="105"/>
+      <c r="D76" s="106"/>
+      <c r="E76" s="106"/>
+      <c r="F76" s="106"/>
+      <c r="G76" s="107"/>
       <c r="H76" s="10"/>
       <c r="I76" s="3"/>
       <c r="J76" s="3"/>
@@ -6369,21 +6350,21 @@
       </c>
       <c r="L76" s="6"/>
       <c r="M76" s="11"/>
-      <c r="N76" s="106"/>
-      <c r="O76" s="104"/>
-      <c r="P76" s="104"/>
-      <c r="Q76" s="104"/>
-      <c r="R76" s="104"/>
-      <c r="S76" s="104"/>
-      <c r="T76" s="104"/>
-      <c r="U76" s="104"/>
-      <c r="V76" s="104"/>
-      <c r="W76" s="104"/>
-      <c r="X76" s="104"/>
-      <c r="Y76" s="104"/>
-      <c r="Z76" s="104"/>
-      <c r="AA76" s="104"/>
-      <c r="AB76" s="105"/>
+      <c r="N76" s="143"/>
+      <c r="O76" s="106"/>
+      <c r="P76" s="106"/>
+      <c r="Q76" s="106"/>
+      <c r="R76" s="106"/>
+      <c r="S76" s="106"/>
+      <c r="T76" s="106"/>
+      <c r="U76" s="106"/>
+      <c r="V76" s="106"/>
+      <c r="W76" s="106"/>
+      <c r="X76" s="106"/>
+      <c r="Y76" s="106"/>
+      <c r="Z76" s="106"/>
+      <c r="AA76" s="106"/>
+      <c r="AB76" s="107"/>
       <c r="AC76" s="10"/>
       <c r="AD76" s="3"/>
       <c r="AE76" s="3"/>
@@ -6540,22 +6521,22 @@
     </row>
     <row r="80" spans="2:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B80" s="3"/>
-      <c r="C80" s="107"/>
-      <c r="D80" s="108"/>
-      <c r="E80" s="108"/>
-      <c r="F80" s="109"/>
+      <c r="C80" s="144"/>
+      <c r="D80" s="134"/>
+      <c r="E80" s="134"/>
+      <c r="F80" s="145"/>
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
       <c r="I80" s="3"/>
       <c r="J80" s="3"/>
-      <c r="K80" s="107"/>
-      <c r="L80" s="108"/>
-      <c r="M80" s="108"/>
-      <c r="N80" s="108"/>
-      <c r="O80" s="108"/>
-      <c r="P80" s="108"/>
-      <c r="Q80" s="108"/>
-      <c r="R80" s="109"/>
+      <c r="K80" s="144"/>
+      <c r="L80" s="134"/>
+      <c r="M80" s="134"/>
+      <c r="N80" s="134"/>
+      <c r="O80" s="134"/>
+      <c r="P80" s="134"/>
+      <c r="Q80" s="134"/>
+      <c r="R80" s="145"/>
       <c r="S80" s="3"/>
       <c r="T80" s="3"/>
       <c r="U80" s="3"/>
@@ -6585,28 +6566,28 @@
     </row>
     <row r="81" spans="2:44" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B81" s="3"/>
-      <c r="C81" s="110" t="s">
+      <c r="C81" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="D81" s="108"/>
-      <c r="E81" s="108"/>
-      <c r="F81" s="109"/>
+      <c r="D81" s="134"/>
+      <c r="E81" s="134"/>
+      <c r="F81" s="145"/>
       <c r="G81" s="8" t="s">
         <v>47</v>
       </c>
       <c r="H81" s="3"/>
       <c r="I81" s="3"/>
       <c r="J81" s="3"/>
-      <c r="K81" s="110" t="s">
+      <c r="K81" s="146" t="s">
         <v>53</v>
       </c>
-      <c r="L81" s="108"/>
-      <c r="M81" s="108"/>
-      <c r="N81" s="108"/>
-      <c r="O81" s="108"/>
-      <c r="P81" s="108"/>
-      <c r="Q81" s="108"/>
-      <c r="R81" s="109"/>
+      <c r="L81" s="134"/>
+      <c r="M81" s="134"/>
+      <c r="N81" s="134"/>
+      <c r="O81" s="134"/>
+      <c r="P81" s="134"/>
+      <c r="Q81" s="134"/>
+      <c r="R81" s="145"/>
       <c r="S81" s="6"/>
       <c r="T81" s="7" t="s">
         <v>47</v>
@@ -49343,16 +49324,35 @@
     </row>
   </sheetData>
   <mergeCells count="55">
-    <mergeCell ref="A2:AA2"/>
-    <mergeCell ref="A3:AA3"/>
-    <mergeCell ref="A4:AA4"/>
-    <mergeCell ref="D6:AA6"/>
-    <mergeCell ref="AC6:AR6"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="D10:AA10"/>
-    <mergeCell ref="AB10:AB11"/>
-    <mergeCell ref="AC10:AD11"/>
+    <mergeCell ref="C76:G76"/>
+    <mergeCell ref="N76:AB76"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="K80:R80"/>
+    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="K81:R81"/>
+    <mergeCell ref="AO14:AP14"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="G16:G18"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="W17:AA17"/>
+    <mergeCell ref="AC17:AC18"/>
+    <mergeCell ref="AD17:AD18"/>
+    <mergeCell ref="AI17:AI18"/>
+    <mergeCell ref="AJ17:AJ18"/>
+    <mergeCell ref="AC14:AF14"/>
+    <mergeCell ref="AG14:AI14"/>
+    <mergeCell ref="AK14:AN14"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="I12:Q12"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="E16:E18"/>
+    <mergeCell ref="F16:F18"/>
+    <mergeCell ref="D14:AA14"/>
+    <mergeCell ref="R12:AA12"/>
+    <mergeCell ref="H17:Q17"/>
+    <mergeCell ref="R17:T17"/>
+    <mergeCell ref="H16:AB16"/>
     <mergeCell ref="AH10:AI11"/>
     <mergeCell ref="AM10:AO11"/>
     <mergeCell ref="R8:AA8"/>
@@ -49369,35 +49369,16 @@
     <mergeCell ref="AF17:AF18"/>
     <mergeCell ref="AG17:AG18"/>
     <mergeCell ref="AH17:AH18"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="I12:Q12"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="E16:E18"/>
-    <mergeCell ref="F16:F18"/>
-    <mergeCell ref="D14:AA14"/>
-    <mergeCell ref="R12:AA12"/>
-    <mergeCell ref="H17:Q17"/>
-    <mergeCell ref="R17:T17"/>
-    <mergeCell ref="H16:AB16"/>
-    <mergeCell ref="AO14:AP14"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="G16:G18"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="W17:AA17"/>
-    <mergeCell ref="AC17:AC18"/>
-    <mergeCell ref="AD17:AD18"/>
-    <mergeCell ref="AI17:AI18"/>
-    <mergeCell ref="AJ17:AJ18"/>
-    <mergeCell ref="AC14:AF14"/>
-    <mergeCell ref="AG14:AI14"/>
-    <mergeCell ref="AK14:AN14"/>
-    <mergeCell ref="C76:G76"/>
-    <mergeCell ref="N76:AB76"/>
-    <mergeCell ref="C80:F80"/>
-    <mergeCell ref="K80:R80"/>
-    <mergeCell ref="C81:F81"/>
-    <mergeCell ref="K81:R81"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="D10:AA10"/>
+    <mergeCell ref="AB10:AB11"/>
+    <mergeCell ref="AC10:AD11"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="A3:AA3"/>
+    <mergeCell ref="A4:AA4"/>
+    <mergeCell ref="D6:AA6"/>
+    <mergeCell ref="AC6:AR6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="CURP - Introduzca el Curp del alumno con 18 dígitos" sqref="G19:G21" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>